<commit_message>
Add ALLMAX Lithium batteries' capacity to tested AAs & AAAs
</commit_message>
<xml_diff>
--- a/hardware/battery-capacity-tests_lithium-ion_AA-AAA.xlsx
+++ b/hardware/battery-capacity-tests_lithium-ion_AA-AAA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mcava\Documents\GitHub\Coding\hardware\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E60155C7-F328-4CB7-AF0B-0381D9B7B9DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF976881-59EB-433E-8707-82E05B752F54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="26010" windowHeight="20985" xr2:uid="{E5D7BF72-F0C5-4096-89C0-8DC37475FB76}"/>
+    <workbookView xWindow="645" yWindow="780" windowWidth="24555" windowHeight="19290" xr2:uid="{E5D7BF72-F0C5-4096-89C0-8DC37475FB76}"/>
   </bookViews>
   <sheets>
     <sheet name="AA Batteries" sheetId="4" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="51">
   <si>
     <t>EBL</t>
   </si>
@@ -194,6 +194,12 @@
   </si>
   <si>
     <t>Lithium Ion</t>
+  </si>
+  <si>
+    <t>ALLMAX</t>
+  </si>
+  <si>
+    <t>Lithium</t>
   </si>
 </sst>
 </file>
@@ -347,18 +353,6 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="dotted">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="164" formatCode="0&quot; mAh&quot;"/>
     </dxf>
     <dxf>
@@ -384,6 +378,18 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="0&quot; mAh&quot;"/>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="dotted">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
     </dxf>
     <dxf>
       <border diagonalUp="0" diagonalDown="0">
@@ -434,28 +440,28 @@
   <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{CBABFE4A-DB4B-478A-A196-6B10725888CE}" name="Battery Brand" dataDxfId="22"/>
     <tableColumn id="2" xr3:uid="{A4C15DEC-98CA-4B4A-AA6D-9D8629196B6D}" name="Form Factor"/>
-    <tableColumn id="18" xr3:uid="{5C2654CB-3147-4CBC-B035-883A9090E4E6}" name="Chemistry" dataDxfId="12"/>
+    <tableColumn id="18" xr3:uid="{5C2654CB-3147-4CBC-B035-883A9090E4E6}" name="Chemistry" dataDxfId="21"/>
     <tableColumn id="3" xr3:uid="{C5D6165E-2DC1-490A-8745-775A230CE959}" name="Plug Loc"/>
     <tableColumn id="4" xr3:uid="{76E5C7FE-A9FC-4892-AA2F-F4BDBC0FE43E}" name="USB Type"/>
     <tableColumn id="5" xr3:uid="{0B30B98B-6A8B-4BC5-AAA4-52D69388E8A1}" name="Splitter Incl."/>
     <tableColumn id="6" xr3:uid="{679FA49F-E3B8-466B-A769-C279FED07A47}" name="Cutoff_x000a_(V)"/>
     <tableColumn id="7" xr3:uid="{0749C5D5-9FE3-4320-A646-E78C6602DB2D}" name="Current_x000a_(A)"/>
-    <tableColumn id="8" xr3:uid="{FC5DC19F-46DB-49F0-B6EB-F8D8DFCC5119}" name="Capacity (mAh)_x000a_(Test #1)" dataDxfId="21"/>
-    <tableColumn id="9" xr3:uid="{2C2758A8-2AF5-47E7-BF85-99A3D8B3BA30}" name="Capacity (mAh)_x000a_(Test #2)" dataDxfId="20"/>
-    <tableColumn id="10" xr3:uid="{33DF939F-2A16-4823-AACA-AC4D2782FCC1}" name="Capacity (mAh)_x000a_(Test #3)" dataDxfId="19"/>
-    <tableColumn id="11" xr3:uid="{DD1EEECD-4600-48C0-A802-DB79834A7A50}" name="Capacity (mAh)_x000a_(Test #4)" dataDxfId="18"/>
-    <tableColumn id="12" xr3:uid="{815B7A98-D189-4530-8370-36E96E9386A8}" name="Capacity (mAh)_x000a_(Averaged)" dataDxfId="17">
+    <tableColumn id="8" xr3:uid="{FC5DC19F-46DB-49F0-B6EB-F8D8DFCC5119}" name="Capacity (mAh)_x000a_(Test #1)" dataDxfId="20"/>
+    <tableColumn id="9" xr3:uid="{2C2758A8-2AF5-47E7-BF85-99A3D8B3BA30}" name="Capacity (mAh)_x000a_(Test #2)" dataDxfId="19"/>
+    <tableColumn id="10" xr3:uid="{33DF939F-2A16-4823-AACA-AC4D2782FCC1}" name="Capacity (mAh)_x000a_(Test #3)" dataDxfId="18"/>
+    <tableColumn id="11" xr3:uid="{DD1EEECD-4600-48C0-A802-DB79834A7A50}" name="Capacity (mAh)_x000a_(Test #4)" dataDxfId="17"/>
+    <tableColumn id="12" xr3:uid="{815B7A98-D189-4530-8370-36E96E9386A8}" name="Capacity (mAh)_x000a_(Averaged)" dataDxfId="16">
       <calculatedColumnFormula>IFERROR(ROUND(AVERAGE(Table35[[#This Row],[Capacity (mAh)
 (Test '#1)]:[Capacity (mAh)
 (Test '#4)]]),0),"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{FB50ABF7-3A80-4E6B-B421-533E61A624AE}" name="Package Quantity" dataDxfId="16"/>
-    <tableColumn id="14" xr3:uid="{BAAC862F-FE09-469C-B505-5B1D17C687E4}" name="Package Price_x000a_($)" dataDxfId="15"/>
-    <tableColumn id="15" xr3:uid="{4DAA5FFD-D836-4119-968C-53A1BFEA75AC}" name="Price per battery_x000a_($)" dataDxfId="14">
+    <tableColumn id="13" xr3:uid="{FB50ABF7-3A80-4E6B-B421-533E61A624AE}" name="Package Quantity" dataDxfId="15"/>
+    <tableColumn id="14" xr3:uid="{BAAC862F-FE09-469C-B505-5B1D17C687E4}" name="Package Price_x000a_($)" dataDxfId="14"/>
+    <tableColumn id="15" xr3:uid="{4DAA5FFD-D836-4119-968C-53A1BFEA75AC}" name="Price per battery_x000a_($)" dataDxfId="13">
       <calculatedColumnFormula>IFERROR(Table35[[#This Row],[Package Price
 ($)]]/Table35[[#This Row],[Package Quantity]],"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{B90ADC68-DA10-4B4A-816B-714216F488CF}" name="Capacity per Dollar (mAh)" dataDxfId="13">
+    <tableColumn id="16" xr3:uid="{B90ADC68-DA10-4B4A-816B-714216F488CF}" name="Capacity per Dollar (mAh)" dataDxfId="12">
       <calculatedColumnFormula>IFERROR(Table35[[#This Row],[Capacity (mAh)
 (Averaged)]]/Table35[[#This Row],[Price per battery
 ($)]],"")</calculatedColumnFormula>
@@ -1301,36 +1307,64 @@
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A9" s="2"/>
+      <c r="A9" s="2" t="s">
+        <v>49</v>
+      </c>
       <c r="B9" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
-      <c r="I9" s="3"/>
-      <c r="J9" s="3"/>
-      <c r="K9" s="3"/>
-      <c r="L9" s="3"/>
-      <c r="M9" s="1" t="str">
+      <c r="C9" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I9" s="3">
+        <v>3236</v>
+      </c>
+      <c r="J9" s="3">
+        <v>3236</v>
+      </c>
+      <c r="K9" s="3">
+        <v>3158</v>
+      </c>
+      <c r="L9" s="3">
+        <v>3170</v>
+      </c>
+      <c r="M9" s="1">
         <f>IFERROR(ROUND(AVERAGE(Table35[[#This Row],[Capacity (mAh)
 (Test '#1)]:[Capacity (mAh)
 (Test '#4)]]),0),"")</f>
-        <v/>
-      </c>
-      <c r="P9" s="11" t="str">
+        <v>3200</v>
+      </c>
+      <c r="N9" s="8">
+        <v>24</v>
+      </c>
+      <c r="O9" s="11">
+        <v>26.99</v>
+      </c>
+      <c r="P9" s="11">
         <f>IFERROR(Table35[[#This Row],[Package Price
 ($)]]/Table35[[#This Row],[Package Quantity]],"")</f>
-        <v/>
-      </c>
-      <c r="Q9" s="1" t="str">
+        <v>1.1245833333333333</v>
+      </c>
+      <c r="Q9" s="1">
         <f>IFERROR(Table35[[#This Row],[Capacity (mAh)
 (Averaged)]]/Table35[[#This Row],[Price per battery
 ($)]],"")</f>
-        <v/>
+        <v>2845.4983327158207</v>
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.25">
@@ -2444,36 +2478,64 @@
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A10" s="2"/>
+      <c r="A10" s="2" t="s">
+        <v>49</v>
+      </c>
       <c r="B10" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
-      <c r="I10" s="3"/>
-      <c r="J10" s="3"/>
-      <c r="K10" s="3"/>
-      <c r="L10" s="3"/>
-      <c r="M10" s="1" t="str">
+        <v>6</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I10" s="3">
+        <v>1201</v>
+      </c>
+      <c r="J10" s="3">
+        <v>1227</v>
+      </c>
+      <c r="K10" s="3">
+        <v>1201</v>
+      </c>
+      <c r="L10" s="3">
+        <v>1209</v>
+      </c>
+      <c r="M10" s="1">
         <f>IFERROR(ROUND(AVERAGE(Table3[[#This Row],[Capacity (mAh)
 (Test '#1)]:[Capacity (mAh)
 (Test '#4)]]),0),"")</f>
-        <v/>
-      </c>
-      <c r="P10" s="11" t="str">
+        <v>1210</v>
+      </c>
+      <c r="N10" s="8">
+        <v>24</v>
+      </c>
+      <c r="O10" s="11">
+        <v>24.99</v>
+      </c>
+      <c r="P10" s="11">
         <f>IFERROR(Table3[[#This Row],[Package Price
 ($)]]/Table3[[#This Row],[Package Quantity]],"")</f>
-        <v/>
-      </c>
-      <c r="Q10" s="1" t="str">
+        <v>1.04125</v>
+      </c>
+      <c r="Q10" s="1">
         <f>IFERROR(Table3[[#This Row],[Capacity (mAh)
 (Averaged)]]/Table3[[#This Row],[Price per battery
 ($)]],"")</f>
-        <v/>
+        <v>1162.0648259303721</v>
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Add Energizer Ultimate Lithium to AA/AAA battery tests
Add Energizer Ultimate Lithium to AA/AAA battery tests
</commit_message>
<xml_diff>
--- a/hardware/battery-capacity-tests_lithium-ion_AA-AAA.xlsx
+++ b/hardware/battery-capacity-tests_lithium-ion_AA-AAA.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mcava\Documents\GitHub\Coding\hardware\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93BC8CBD-FFBB-498B-AA68-9E0722722326}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37644B9F-22A9-4716-B303-DF7DAC017697}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3510" yWindow="3510" windowWidth="38700" windowHeight="15345" xr2:uid="{E5D7BF72-F0C5-4096-89C0-8DC37475FB76}"/>
+    <workbookView xWindow="3900" yWindow="3900" windowWidth="38700" windowHeight="15345" xr2:uid="{E5D7BF72-F0C5-4096-89C0-8DC37475FB76}"/>
   </bookViews>
   <sheets>
     <sheet name="AA Batteries" sheetId="4" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="55">
   <si>
     <t>EBL</t>
   </si>
@@ -134,9 +134,6 @@
   </si>
   <si>
     <t>6. Press "OK" to confirm the cutoff voltage and the HW-586 will run until the battery reaches 0.8V</t>
-  </si>
-  <si>
-    <t>e-CIRCUIT</t>
   </si>
   <si>
     <t>7. Once test is complete, the HW-586 will bleak rapidly, displaying the "Ah" (Amp-hours) result - Save this into desired spreadsheet or other record keeping location</t>
@@ -212,6 +209,12 @@
   <si>
     <t>Capacity (Claimed)
 (mAh)</t>
+  </si>
+  <si>
+    <t>ENERGIZER ULTIMATE</t>
+  </si>
+  <si>
+    <t>E-CIRCUIT</t>
   </si>
 </sst>
 </file>
@@ -965,7 +968,7 @@
   <dimension ref="A1:T25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.140625" style="7" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.42578125" style="7" customWidth="1"/>
     <col min="2" max="2" width="9.140625" style="7"/>
     <col min="3" max="3" width="12.28515625" style="7" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.140625" style="16" bestFit="1" customWidth="1"/>
@@ -993,13 +996,13 @@
         <v>24</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>8</v>
@@ -1011,51 +1014,51 @@
         <v>15</v>
       </c>
       <c r="I1" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="J1" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="K1" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="L1" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="M1" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="N1" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="O1" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="P1" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q1" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="R1" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="S1" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="T1" s="8" t="s">
         <v>42</v>
-      </c>
-      <c r="K1" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="L1" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="M1" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="N1" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="O1" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="P1" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="Q1" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="R1" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="S1" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="T1" s="8" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>32</v>
+        <v>54</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>5</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>19</v>
@@ -1129,7 +1132,7 @@
         <v>5</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D3" s="4">
         <v>3300</v>
@@ -1201,7 +1204,7 @@
         <v>5</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D4" s="4">
         <v>2600</v>
@@ -1275,7 +1278,7 @@
         <v>5</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D5" s="4">
         <v>2600</v>
@@ -1349,7 +1352,7 @@
         <v>5</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D6" s="4">
         <v>4612</v>
@@ -1423,7 +1426,7 @@
         <v>5</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D7" s="4">
         <v>2960</v>
@@ -1497,7 +1500,7 @@
         <v>5</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D8" s="4">
         <v>3300</v>
@@ -1571,7 +1574,7 @@
         <v>5</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D9" s="4">
         <v>3500</v>
@@ -1639,13 +1642,13 @@
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B10" s="6" t="s">
         <v>5</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D10" s="4">
         <v>4800</v>
@@ -1712,45 +1715,77 @@
       </c>
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A11" s="6"/>
+      <c r="A11" s="6" t="s">
+        <v>53</v>
+      </c>
       <c r="B11" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="C11" s="6"/>
-      <c r="D11" s="4"/>
-      <c r="E11" s="12"/>
-      <c r="F11" s="6"/>
-      <c r="G11" s="6"/>
-      <c r="H11" s="6"/>
-      <c r="I11" s="6"/>
-      <c r="J11" s="6"/>
-      <c r="K11" s="13"/>
-      <c r="L11" s="13"/>
-      <c r="M11" s="13"/>
-      <c r="N11" s="13"/>
-      <c r="O11" s="3" t="str">
+      <c r="C11" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D11" s="4">
+        <v>4500</v>
+      </c>
+      <c r="E11" s="12">
+        <v>1</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I11" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="J11" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="K11" s="13">
+        <v>3318</v>
+      </c>
+      <c r="L11" s="13">
+        <v>3441</v>
+      </c>
+      <c r="M11" s="13">
+        <v>3493</v>
+      </c>
+      <c r="N11" s="13">
+        <v>3511</v>
+      </c>
+      <c r="O11" s="3">
         <f>IFERROR(ROUND(AVERAGE(Table35[[#This Row],[Capacity (mAh)
 (Test '#1)]:[Capacity (mAh)
 (Test '#4)]]),0),"")</f>
-        <v/>
-      </c>
-      <c r="P11" s="3" t="str">
+        <v>3441</v>
+      </c>
+      <c r="P11" s="3">
         <f>IF(OR(ISBLANK(Table35[[#This Row],[Capacity (Claimed)
 (mWh)]]),(Table35[[#This Row],[Capacity (Claimed)
 (mWh)]]="-")),"-",(Table35[[#This Row],[Capacity (Claimed)
 (mWh)]]/1.5))</f>
-        <v>-</v>
-      </c>
-      <c r="S11" s="15" t="str">
+        <v>3000</v>
+      </c>
+      <c r="Q11" s="14">
+        <v>8</v>
+      </c>
+      <c r="R11" s="15">
+        <v>15.99</v>
+      </c>
+      <c r="S11" s="15">
         <f>IFERROR(Table35[[#This Row],[Package Price
 ($)]]/Table35[[#This Row],[Pkg Qty]],"")</f>
-        <v/>
-      </c>
-      <c r="T11" s="3" t="str">
+        <v>1.99875</v>
+      </c>
+      <c r="T11" s="3">
         <f>IFERROR(Table35[[#This Row],[Capacity (mAh)
 (Averaged)]]/Table35[[#This Row],[Price per battery
 ($)]],"")</f>
-        <v/>
+        <v>1721.5759849906192</v>
       </c>
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.25">
@@ -2342,7 +2377,7 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="O2:P25">
+  <conditionalFormatting sqref="O2:O25">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -2367,7 +2402,7 @@
   <dimension ref="A1:T25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.140625" style="7" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.42578125" style="7" customWidth="1"/>
     <col min="2" max="2" width="9.140625" style="7"/>
     <col min="3" max="3" width="12.28515625" style="7" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.140625" style="16" bestFit="1" customWidth="1"/>
@@ -2395,13 +2430,13 @@
         <v>24</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>8</v>
@@ -2413,51 +2448,51 @@
         <v>15</v>
       </c>
       <c r="I1" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="J1" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="K1" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="L1" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="M1" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="N1" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="O1" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="P1" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q1" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="R1" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="S1" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="T1" s="8" t="s">
         <v>42</v>
-      </c>
-      <c r="K1" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="L1" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="M1" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="N1" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="O1" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="P1" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="Q1" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="R1" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="S1" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="T1" s="8" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>32</v>
+        <v>54</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>19</v>
@@ -2531,7 +2566,7 @@
         <v>6</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D3" s="4">
         <v>550</v>
@@ -2605,7 +2640,7 @@
         <v>6</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D4" s="4">
         <v>750</v>
@@ -2679,7 +2714,7 @@
         <v>6</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D5" s="4">
         <v>900</v>
@@ -2753,7 +2788,7 @@
         <v>6</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D6" s="4">
         <v>1875</v>
@@ -2821,13 +2856,13 @@
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D7" s="4">
         <v>1650</v>
@@ -2901,7 +2936,7 @@
         <v>6</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D8" s="4">
         <v>1875</v>
@@ -2975,7 +3010,7 @@
         <v>6</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D9" s="4">
         <v>1100</v>
@@ -3043,13 +3078,13 @@
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B10" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D10" s="4">
         <v>1800</v>
@@ -3747,7 +3782,7 @@
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
-  <conditionalFormatting sqref="O2:P25">
+  <conditionalFormatting sqref="O2:O25">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -3813,7 +3848,7 @@
     </row>
     <row r="8" spans="1:1" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9" spans="1:1" ht="22.5" customHeight="1" x14ac:dyDescent="0.3"/>

</xml_diff>